<commit_message>
Main edit - waterbird script - deleted old code (not useful) and write code for generalised linear models for waterbird analysis
</commit_message>
<xml_diff>
--- a/raw/flows_floods_summary_forR.xlsx
+++ b/raw/flows_floods_summary_forR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/cumbung_assessment/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="297" documentId="8_{FD27E311-2AB5-4611-BE74-E4F4C6E3F023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF0AAEFB-B4DE-4857-A6AC-C1618279A98B}"/>
+  <xr:revisionPtr revIDLastSave="302" documentId="8_{FD27E311-2AB5-4611-BE74-E4F4C6E3F023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92B7531C-333B-420D-9271-8BC2EA5894FB}"/>
   <bookViews>
-    <workbookView xWindow="36" yWindow="36" windowWidth="12456" windowHeight="13668" firstSheet="13" activeTab="13" xr2:uid="{74D5E0EF-1549-41B2-9103-C2DB8A5CCD57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" firstSheet="4" activeTab="7" xr2:uid="{74D5E0EF-1549-41B2-9103-C2DB8A5CCD57}"/>
   </bookViews>
   <sheets>
     <sheet name="all_5yr" sheetId="18" r:id="rId1"/>
@@ -13350,8 +13350,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77AE11BE-A164-43B3-BC5B-6B8B2CA5EFCA}">
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="8.88671875" style="3"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -14441,7 +14444,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2009</v>
       </c>
@@ -14458,7 +14461,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2010</v>
       </c>
@@ -14474,8 +14477,9 @@
       <c r="E66">
         <v>365</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H66" s="3"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>2011</v>
       </c>
@@ -14491,8 +14495,9 @@
       <c r="E67">
         <v>365</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2012</v>
       </c>
@@ -14508,8 +14513,9 @@
       <c r="E68">
         <v>366</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H68" s="3"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>2013</v>
       </c>
@@ -14525,8 +14531,9 @@
       <c r="E69">
         <v>365</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H69" s="3"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>2014</v>
       </c>
@@ -14542,8 +14549,9 @@
       <c r="E70">
         <v>365</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H70" s="3"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>2015</v>
       </c>
@@ -14559,8 +14567,9 @@
       <c r="E71">
         <v>364</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>2016</v>
       </c>
@@ -14576,8 +14585,9 @@
       <c r="E72">
         <v>366</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H72" s="3"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>2017</v>
       </c>
@@ -14593,8 +14603,9 @@
       <c r="E73">
         <v>365</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H73" s="3"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>2018</v>
       </c>
@@ -14610,8 +14621,9 @@
       <c r="E74">
         <v>365</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H74" s="3"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>2019</v>
       </c>
@@ -14627,8 +14639,9 @@
       <c r="E75">
         <v>365</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H75" s="3"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>2020</v>
       </c>
@@ -14644,8 +14657,9 @@
       <c r="E76">
         <v>366</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H76" s="3"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>2021</v>
       </c>
@@ -14661,6 +14675,7 @@
       <c r="E77">
         <v>128</v>
       </c>
+      <c r="H77" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>